<commit_message>
Fix nom synthese PDF
</commit_message>
<xml_diff>
--- a/cv/tableau_complete (1).xlsx
+++ b/cv/tableau_complete (1).xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\portfolio\ Portfolio Website\cv\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19368" windowHeight="10332"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -142,48 +142,283 @@
     <t>Mésure de la visibilité de l'organisation via les données Google Maps et Search</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">SESSION </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="20"/>
+    <t>S1-S4</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     S3</t>
+  </si>
+  <si>
+    <t>05/01/2026 Au 13/02/2026</t>
+  </si>
+  <si>
+    <t>12/05/2025 Au 27/06/2025</t>
+  </si>
+  <si>
+    <r>
+      <t>Apprentissage NestJS, React, nouvelles</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> technos</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Planification,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> méthodode</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> agile, analyse des écarts</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Utilisation du standard Oauth 2,0 et gestion des ID </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>clients</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> sécurisés</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Planification des</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> activités, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>analyse</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>des</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> objectifs et comptes rendus </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>hebdomadaires</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Réalisations des tests (débogage erreur 400) et </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">déploiement de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>l'application en local (Live Server) pour les utilisateurs</t>
+    </r>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>AP-Gestion des équipes sportives numériques apparteneant a</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> une mairie</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>AP3-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">rojet GSB (C#) </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>dévéloppement</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> d'une IHM Windows Form avec connexion à une base de données</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>AP-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>cybersécurité</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (analyse d'une application web vulnérable et contre mésure)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Prise de connexion du cahier de charge</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
         <color rgb="FFFF0000"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>2026</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Centre de formation :</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Lycée Carcouët</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Adresse URL du portfolio : </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>https://krou-eric.github.io</t>
+      <t xml:space="preserve"> </t>
     </r>
   </si>
   <si>
@@ -209,7 +444,7 @@
       <rPr>
         <b/>
         <sz val="18"/>
-        <color rgb="FFFF0000"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -218,13 +453,28 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">SESSION </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="20"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2026</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">NOM et prénom : </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="18"/>
-        <color rgb="FFFF0000"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
@@ -233,298 +483,39 @@
   </si>
   <si>
     <r>
-      <t>TP-mobile</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (pas suffisement précis, développe cet item)</t>
-    </r>
-  </si>
-  <si>
-    <t>S1-S4</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     S3</t>
-  </si>
-  <si>
-    <t>05/01/2026 Au 13/02/2026</t>
-  </si>
-  <si>
-    <t>12/05/2025 Au 27/06/2025</t>
-  </si>
-  <si>
-    <r>
-      <t>Apprentissage NestJS, React, nouvelles</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
+      <t>Centre de formation :</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
         <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> technos</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Planification,</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
+      <t xml:space="preserve"> Lycée Carcouët</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Adresse URL du portfolio : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
         <color theme="1"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> méthodode</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> agile, analyse des écarts</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Utilisation du standard Oauth 2,0 et gestion des ID </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>clients</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> sécurisés</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Planification des</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> activités, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>analyse</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>des</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> objectifs et comptes rendus </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>hebdomadaires</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Réalisations des tests (débogage erreur 400) et </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">déploiement de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>l'application en local (Live Server) pour les utilisateurs</t>
-    </r>
-  </si>
-  <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>AP-Gestion des équipes sportives numériques apparteneant a</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> une mairie</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>AP3-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>P</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">rojet GSB (C#) </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>dévéloppement</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> d'une IHM Windows Form avec connexion à une base de données</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>AP-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>cybersécurité</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (analyse d'une application web vulnérable et contre mésure)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Prise de connexion du cahier de charge</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
+      <t>https://krou-eric.github.io</t>
+    </r>
+  </si>
+  <si>
+    <t>S4</t>
+  </si>
+  <si>
+    <t>TP-mobile</t>
   </si>
 </sst>
 </file>
@@ -616,20 +607,6 @@
     </font>
     <font>
       <b/>
-      <sz val="20"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="18"/>
       <name val="Wingdings"/>
       <charset val="2"/>
@@ -665,6 +642,20 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -1056,7 +1047,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1133,23 +1124,38 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1175,35 +1181,17 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1525,56 +1513,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.9" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="50"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="31"/>
     </row>
     <row r="2" spans="1:13" ht="41.1" customHeight="1" thickBot="1">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="3" spans="1:13" ht="39.9" customHeight="1">
-      <c r="A3" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="36" t="s">
+      <c r="A3" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="42"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="38"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.9" customHeight="1">
-      <c r="A4" s="48" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
+      <c r="A4" s="54" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
@@ -1582,26 +1570,26 @@
         <v>4</v>
       </c>
       <c r="H4" s="26" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A5" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="35"/>
+      <c r="A5" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="40"/>
     </row>
     <row r="6" spans="1:13" ht="90" customHeight="1">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="44" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1624,8 +1612,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1">
-      <c r="A7" s="44"/>
-      <c r="B7" s="40"/>
+      <c r="A7" s="49"/>
+      <c r="B7" s="45"/>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
@@ -1646,23 +1634,23 @@
       </c>
     </row>
     <row r="8" spans="1:13" s="2" customFormat="1" ht="17.399999999999999" customHeight="1">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="42"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="47"/>
     </row>
     <row r="9" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A9" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>41</v>
+        <v>47</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>35</v>
       </c>
       <c r="C9" s="22" t="s">
         <v>20</v>
@@ -1672,7 +1660,7 @@
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13"/>
-      <c r="G9" s="51" t="s">
+      <c r="G9" s="27" t="s">
         <v>20</v>
       </c>
       <c r="H9" s="25" t="s">
@@ -1681,10 +1669,10 @@
     </row>
     <row r="10" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A10" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B10" s="52" t="s">
-        <v>50</v>
+        <v>45</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>44</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
@@ -1703,8 +1691,8 @@
       <c r="A11" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="52" t="s">
-        <v>49</v>
+      <c r="B11" s="28" t="s">
+        <v>43</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -1712,7 +1700,7 @@
         <v>20</v>
       </c>
       <c r="F11" s="13"/>
-      <c r="G11" s="51" t="s">
+      <c r="G11" s="27" t="s">
         <v>20</v>
       </c>
       <c r="H11" s="25" t="s">
@@ -1721,10 +1709,10 @@
     </row>
     <row r="12" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A12" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="52" t="s">
-        <v>40</v>
+        <v>46</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>34</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -1743,8 +1731,8 @@
       <c r="A13" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="52" t="s">
-        <v>39</v>
+      <c r="B13" s="28" t="s">
+        <v>33</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
@@ -1759,9 +1747,11 @@
     </row>
     <row r="14" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A14" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="27"/>
+        <v>55</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>54</v>
+      </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
@@ -1777,8 +1767,8 @@
       <c r="A15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="52" t="s">
-        <v>39</v>
+      <c r="B15" s="28" t="s">
+        <v>33</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
@@ -1790,23 +1780,23 @@
       </c>
     </row>
     <row r="16" spans="1:13" s="2" customFormat="1" ht="17.399999999999999" customHeight="1">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="32"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="34"/>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A17" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="54" t="s">
-        <v>43</v>
+      <c r="B17" s="51" t="s">
+        <v>37</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -1823,9 +1813,9 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" s="46"/>
+        <v>39</v>
+      </c>
+      <c r="B18" s="52"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
@@ -1839,7 +1829,7 @@
       <c r="A19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="46"/>
+      <c r="B19" s="52"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
@@ -1851,9 +1841,9 @@
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A20" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="46"/>
+        <v>38</v>
+      </c>
+      <c r="B20" s="52"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
@@ -1867,7 +1857,7 @@
       <c r="A21" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="46"/>
+      <c r="B21" s="52"/>
       <c r="C21" s="13"/>
       <c r="D21" s="17" t="s">
         <v>20</v>
@@ -1879,9 +1869,9 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A22" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="47"/>
+        <v>48</v>
+      </c>
+      <c r="B22" s="53"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
@@ -1892,23 +1882,23 @@
       <c r="H22" s="14"/>
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" ht="17.399999999999999" customHeight="1">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="32"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="34"/>
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A24" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="55" t="s">
-        <v>42</v>
+      <c r="B24" s="35" t="s">
+        <v>36</v>
       </c>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
@@ -1923,8 +1913,8 @@
       <c r="A25" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="51" t="s">
+      <c r="B25" s="36"/>
+      <c r="C25" s="27" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="17" t="s">
@@ -1937,9 +1927,9 @@
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A26" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="28"/>
+        <v>42</v>
+      </c>
+      <c r="B26" s="36"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
@@ -1953,7 +1943,7 @@
       <c r="A27" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="28"/>
+      <c r="B27" s="36"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
       <c r="E27" s="13"/>
@@ -1965,9 +1955,9 @@
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A28" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="28"/>
+        <v>41</v>
+      </c>
+      <c r="B28" s="36"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
@@ -1981,7 +1971,7 @@
       <c r="A29" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="28"/>
+      <c r="B29" s="36"/>
       <c r="C29" s="17"/>
       <c r="D29" s="13"/>
       <c r="E29" s="17" t="s">
@@ -1993,9 +1983,9 @@
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A30" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="B30" s="29"/>
+        <v>40</v>
+      </c>
+      <c r="B30" s="37"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
Ajout cahier des charges Google Analytics
</commit_message>
<xml_diff>
--- a/cv/tableau_complete (1).xlsx
+++ b/cv/tableau_complete (1).xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="55">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -148,9 +148,6 @@
     <t>S3</t>
   </si>
   <si>
-    <t xml:space="preserve">     S3</t>
-  </si>
-  <si>
     <t>05/01/2026 Au 13/02/2026</t>
   </si>
   <si>
@@ -515,7 +512,7 @@
     <t>S4</t>
   </si>
   <si>
-    <t>TP-mobile</t>
+    <t>TP- Développement d'une application Android</t>
   </si>
 </sst>
 </file>
@@ -525,7 +522,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -657,6 +654,18 @@
       <b/>
       <sz val="20"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="24"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1047,7 +1056,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1091,12 +1100,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1132,9 +1135,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1192,6 +1192,24 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1513,83 +1531,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.9" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="28"/>
+    </row>
+    <row r="2" spans="1:13" ht="41.1" customHeight="1" thickBot="1">
+      <c r="A2" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+    </row>
+    <row r="3" spans="1:13" ht="39.9" customHeight="1">
+      <c r="A3" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="31"/>
-    </row>
-    <row r="2" spans="1:13" ht="41.1" customHeight="1" thickBot="1">
-      <c r="A2" s="30" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-    </row>
-    <row r="3" spans="1:13" ht="39.9" customHeight="1">
-      <c r="A3" s="50" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="41" t="s">
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="42"/>
-      <c r="H3" s="43"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="40"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.9" customHeight="1">
-      <c r="A4" s="54" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="34"/>
+      <c r="A4" s="51" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
       <c r="F4" s="11" t="s">
         <v>3</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="26" t="s">
-        <v>49</v>
+      <c r="H4" s="24" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A5" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="40"/>
+      <c r="A5" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:13" ht="90" customHeight="1">
-      <c r="A6" s="48" t="s">
+      <c r="A6" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="41" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1612,21 +1630,21 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1">
-      <c r="A7" s="49"/>
-      <c r="B7" s="45"/>
-      <c r="C7" s="19" t="s">
+      <c r="A7" s="46"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="17" t="s">
         <v>17</v>
       </c>
       <c r="H7" s="8" t="s">
@@ -1634,95 +1652,95 @@
       </c>
     </row>
     <row r="8" spans="1:13" s="2" customFormat="1" ht="17.399999999999999" customHeight="1">
-      <c r="A8" s="46" t="s">
+      <c r="A8" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="47"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="44"/>
     </row>
     <row r="9" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A9" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>20</v>
       </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13"/>
-      <c r="G9" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="25" t="s">
+      <c r="G9" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A10" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="28" t="s">
         <v>44</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>43</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
-      <c r="E10" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="22" t="s">
+      <c r="E10" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="20" t="s">
         <v>20</v>
       </c>
       <c r="H10" s="14"/>
     </row>
     <row r="11" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="28" t="s">
-        <v>43</v>
+      <c r="B11" s="26" t="s">
+        <v>42</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="22" t="s">
+      <c r="E11" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F11" s="13"/>
-      <c r="G11" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="25" t="s">
+      <c r="G11" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A12" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="26" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
-      <c r="E12" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="22" t="s">
+      <c r="E12" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="20" t="s">
         <v>20</v>
       </c>
       <c r="H12" s="14"/>
@@ -1731,34 +1749,34 @@
       <c r="A13" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="26" t="s">
         <v>33</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
-      <c r="H13" s="23" t="s">
+      <c r="H13" s="21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:13" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A14" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B14" s="28" t="s">
         <v>54</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>53</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
-      <c r="F14" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="22" t="s">
+      <c r="F14" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="20" t="s">
         <v>20</v>
       </c>
       <c r="H14" s="14"/>
@@ -1767,7 +1785,7 @@
       <c r="A15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="26" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="13"/>
@@ -1775,51 +1793,51 @@
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
-      <c r="H15" s="23" t="s">
+      <c r="H15" s="21" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:13" s="2" customFormat="1" ht="17.399999999999999" customHeight="1">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="34"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="31"/>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A17" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="51" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="G17" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H17" s="18"/>
+      <c r="B17" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="16"/>
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="52"/>
+        <v>38</v>
+      </c>
+      <c r="B18" s="49"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="15" t="s">
         <v>20</v>
       </c>
       <c r="G18" s="13"/>
@@ -1829,27 +1847,27 @@
       <c r="A19" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="52"/>
+      <c r="B19" s="49"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
-      <c r="G19" s="17" t="s">
+      <c r="G19" s="15" t="s">
         <v>20</v>
       </c>
       <c r="H19" s="14"/>
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A20" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" s="52"/>
+        <v>37</v>
+      </c>
+      <c r="B20" s="49"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="16" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1857,9 +1875,9 @@
       <c r="A21" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="52"/>
+      <c r="B21" s="49"/>
       <c r="C21" s="13"/>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="15" t="s">
         <v>20</v>
       </c>
       <c r="E21" s="13"/>
@@ -1869,131 +1887,131 @@
     </row>
     <row r="22" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A22" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" s="53"/>
+        <v>47</v>
+      </c>
+      <c r="B22" s="50"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
-      <c r="F22" s="24" t="s">
+      <c r="F22" s="22" t="s">
         <v>20</v>
       </c>
       <c r="G22" s="13"/>
       <c r="H22" s="14"/>
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" ht="17.399999999999999" customHeight="1">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="34"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="31"/>
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A24" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H24" s="18"/>
+      <c r="B24" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H24" s="16"/>
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A25" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="14"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="54"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="55"/>
     </row>
     <row r="26" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A26" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B26" s="36"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H26" s="14"/>
+        <v>41</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="54"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" s="55"/>
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A27" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="18" t="s">
+      <c r="B27" s="33"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="16" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A28" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B28" s="36"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="13"/>
-      <c r="H28" s="14"/>
+        <v>40</v>
+      </c>
+      <c r="B28" s="33"/>
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="54"/>
+      <c r="H28" s="55"/>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A29" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="36"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="14"/>
+      <c r="B29" s="33"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="55"/>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A30" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="16"/>
+        <v>39</v>
+      </c>
+      <c r="B30" s="34"/>
+      <c r="C30" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="57"/>
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" ht="13.95" customHeight="1">
       <c r="A31" s="5"/>

</xml_diff>